<commit_message>
I had to update the dilution factors for all these results because we found out they were tested 25X more concentrated than needed.
</commit_message>
<xml_diff>
--- a/raw/processedSamples/20260512_r2_SG_USDA-Blood_Nano-QuIC.xlsx
+++ b/raw/processedSamples/20260512_r2_SG_USDA-Blood_Nano-QuIC.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MNPRO\Desktop\RT-QuIC Data\Sarah's RT-QuIC Data\2026\20260512_r2_SG_USDA-Blood_Nano-QuIC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rowde002\Documents\Projects\usda-validation\raw\processedSamples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C96871C6-EA2F-4986-B0CE-C2AA812F234C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00319E17-3730-443F-A8B8-350E3098AE98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5130" yWindow="540" windowWidth="21600" windowHeight="13980" xr2:uid="{AE8526AD-1B67-495C-ABC3-68E59956E741}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AE8526AD-1B67-495C-ABC3-68E59956E741}"/>
   </bookViews>
   <sheets>
     <sheet name="Microplate Cycle 1 (0 h)" sheetId="2" r:id="rId1"/>
@@ -1639,37 +1639,37 @@
         <v>1000</v>
       </c>
       <c r="C27" s="12">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="D27" s="12">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="E27" s="12">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="F27" s="12">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="G27" s="12">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="H27" s="12">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="I27" s="12">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="J27" s="12">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="K27" s="12">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="L27" s="12">
-        <v>100</v>
-      </c>
-      <c r="M27" s="13">
-        <v>100</v>
+        <v>4</v>
+      </c>
+      <c r="M27" s="12">
+        <v>4</v>
       </c>
       <c r="O27" s="21"/>
     </row>
@@ -1680,38 +1680,38 @@
       <c r="B28" s="5">
         <v>1000</v>
       </c>
-      <c r="C28" s="14">
-        <v>100</v>
-      </c>
-      <c r="D28" s="14">
-        <v>100</v>
-      </c>
-      <c r="E28" s="14">
-        <v>100</v>
-      </c>
-      <c r="F28" s="14">
-        <v>100</v>
-      </c>
-      <c r="G28" s="14">
-        <v>100</v>
-      </c>
-      <c r="H28" s="14">
-        <v>100</v>
-      </c>
-      <c r="I28" s="14">
-        <v>100</v>
-      </c>
-      <c r="J28" s="14">
-        <v>100</v>
-      </c>
-      <c r="K28" s="14">
-        <v>100</v>
-      </c>
-      <c r="L28" s="14">
-        <v>100</v>
-      </c>
-      <c r="M28" s="15">
-        <v>100</v>
+      <c r="C28" s="12">
+        <v>4</v>
+      </c>
+      <c r="D28" s="12">
+        <v>4</v>
+      </c>
+      <c r="E28" s="12">
+        <v>4</v>
+      </c>
+      <c r="F28" s="12">
+        <v>4</v>
+      </c>
+      <c r="G28" s="12">
+        <v>4</v>
+      </c>
+      <c r="H28" s="12">
+        <v>4</v>
+      </c>
+      <c r="I28" s="12">
+        <v>4</v>
+      </c>
+      <c r="J28" s="12">
+        <v>4</v>
+      </c>
+      <c r="K28" s="12">
+        <v>4</v>
+      </c>
+      <c r="L28" s="12">
+        <v>4</v>
+      </c>
+      <c r="M28" s="12">
+        <v>4</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
@@ -1721,38 +1721,38 @@
       <c r="B29" s="5">
         <v>1000</v>
       </c>
-      <c r="C29" s="14">
-        <v>100</v>
-      </c>
-      <c r="D29" s="14">
-        <v>100</v>
-      </c>
-      <c r="E29" s="14">
-        <v>100</v>
-      </c>
-      <c r="F29" s="14">
-        <v>100</v>
-      </c>
-      <c r="G29" s="14">
-        <v>100</v>
-      </c>
-      <c r="H29" s="14">
-        <v>100</v>
-      </c>
-      <c r="I29" s="14">
-        <v>100</v>
-      </c>
-      <c r="J29" s="14">
-        <v>100</v>
-      </c>
-      <c r="K29" s="14">
-        <v>100</v>
-      </c>
-      <c r="L29" s="14">
-        <v>100</v>
-      </c>
-      <c r="M29" s="15">
-        <v>100</v>
+      <c r="C29" s="12">
+        <v>4</v>
+      </c>
+      <c r="D29" s="12">
+        <v>4</v>
+      </c>
+      <c r="E29" s="12">
+        <v>4</v>
+      </c>
+      <c r="F29" s="12">
+        <v>4</v>
+      </c>
+      <c r="G29" s="12">
+        <v>4</v>
+      </c>
+      <c r="H29" s="12">
+        <v>4</v>
+      </c>
+      <c r="I29" s="12">
+        <v>4</v>
+      </c>
+      <c r="J29" s="12">
+        <v>4</v>
+      </c>
+      <c r="K29" s="12">
+        <v>4</v>
+      </c>
+      <c r="L29" s="12">
+        <v>4</v>
+      </c>
+      <c r="M29" s="12">
+        <v>4</v>
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
@@ -1762,38 +1762,38 @@
       <c r="B30" s="5">
         <v>1000</v>
       </c>
-      <c r="C30" s="14">
-        <v>100</v>
-      </c>
-      <c r="D30" s="14">
-        <v>100</v>
-      </c>
-      <c r="E30" s="14">
-        <v>100</v>
-      </c>
-      <c r="F30" s="14">
-        <v>100</v>
-      </c>
-      <c r="G30" s="14">
-        <v>100</v>
-      </c>
-      <c r="H30" s="14">
-        <v>100</v>
-      </c>
-      <c r="I30" s="14">
-        <v>100</v>
-      </c>
-      <c r="J30" s="14">
-        <v>100</v>
-      </c>
-      <c r="K30" s="14">
-        <v>100</v>
-      </c>
-      <c r="L30" s="14">
-        <v>100</v>
-      </c>
-      <c r="M30" s="15">
-        <v>100</v>
+      <c r="C30" s="12">
+        <v>4</v>
+      </c>
+      <c r="D30" s="12">
+        <v>4</v>
+      </c>
+      <c r="E30" s="12">
+        <v>4</v>
+      </c>
+      <c r="F30" s="12">
+        <v>4</v>
+      </c>
+      <c r="G30" s="12">
+        <v>4</v>
+      </c>
+      <c r="H30" s="12">
+        <v>4</v>
+      </c>
+      <c r="I30" s="12">
+        <v>4</v>
+      </c>
+      <c r="J30" s="12">
+        <v>4</v>
+      </c>
+      <c r="K30" s="12">
+        <v>4</v>
+      </c>
+      <c r="L30" s="12">
+        <v>4</v>
+      </c>
+      <c r="M30" s="12">
+        <v>4</v>
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
@@ -1803,38 +1803,38 @@
       <c r="B31" s="5">
         <v>1000</v>
       </c>
-      <c r="C31" s="14">
-        <v>100</v>
-      </c>
-      <c r="D31" s="14">
-        <v>100</v>
-      </c>
-      <c r="E31" s="14">
-        <v>100</v>
-      </c>
-      <c r="F31" s="14">
-        <v>100</v>
-      </c>
-      <c r="G31" s="14">
-        <v>100</v>
-      </c>
-      <c r="H31" s="14">
-        <v>100</v>
-      </c>
-      <c r="I31" s="14">
-        <v>100</v>
-      </c>
-      <c r="J31" s="14">
-        <v>100</v>
-      </c>
-      <c r="K31" s="14">
-        <v>100</v>
-      </c>
-      <c r="L31" s="14">
-        <v>100</v>
-      </c>
-      <c r="M31" s="15">
-        <v>100</v>
+      <c r="C31" s="12">
+        <v>4</v>
+      </c>
+      <c r="D31" s="12">
+        <v>4</v>
+      </c>
+      <c r="E31" s="12">
+        <v>4</v>
+      </c>
+      <c r="F31" s="12">
+        <v>4</v>
+      </c>
+      <c r="G31" s="12">
+        <v>4</v>
+      </c>
+      <c r="H31" s="12">
+        <v>4</v>
+      </c>
+      <c r="I31" s="12">
+        <v>4</v>
+      </c>
+      <c r="J31" s="12">
+        <v>4</v>
+      </c>
+      <c r="K31" s="12">
+        <v>4</v>
+      </c>
+      <c r="L31" s="12">
+        <v>4</v>
+      </c>
+      <c r="M31" s="12">
+        <v>4</v>
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
@@ -1844,38 +1844,38 @@
       <c r="B32" s="5">
         <v>1000</v>
       </c>
-      <c r="C32" s="14">
-        <v>100</v>
-      </c>
-      <c r="D32" s="14">
-        <v>100</v>
-      </c>
-      <c r="E32" s="14">
-        <v>100</v>
-      </c>
-      <c r="F32" s="14">
-        <v>100</v>
-      </c>
-      <c r="G32" s="14">
-        <v>100</v>
-      </c>
-      <c r="H32" s="14">
-        <v>100</v>
-      </c>
-      <c r="I32" s="14">
-        <v>100</v>
-      </c>
-      <c r="J32" s="14">
-        <v>100</v>
-      </c>
-      <c r="K32" s="14">
-        <v>100</v>
-      </c>
-      <c r="L32" s="14">
-        <v>100</v>
-      </c>
-      <c r="M32" s="15">
-        <v>100</v>
+      <c r="C32" s="12">
+        <v>4</v>
+      </c>
+      <c r="D32" s="12">
+        <v>4</v>
+      </c>
+      <c r="E32" s="12">
+        <v>4</v>
+      </c>
+      <c r="F32" s="12">
+        <v>4</v>
+      </c>
+      <c r="G32" s="12">
+        <v>4</v>
+      </c>
+      <c r="H32" s="12">
+        <v>4</v>
+      </c>
+      <c r="I32" s="12">
+        <v>4</v>
+      </c>
+      <c r="J32" s="12">
+        <v>4</v>
+      </c>
+      <c r="K32" s="12">
+        <v>4</v>
+      </c>
+      <c r="L32" s="12">
+        <v>4</v>
+      </c>
+      <c r="M32" s="12">
+        <v>4</v>
       </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.25">
@@ -1885,38 +1885,38 @@
       <c r="B33" s="5">
         <v>1000</v>
       </c>
-      <c r="C33" s="14">
-        <v>100</v>
-      </c>
-      <c r="D33" s="14">
-        <v>100</v>
-      </c>
-      <c r="E33" s="14">
-        <v>100</v>
-      </c>
-      <c r="F33" s="14">
-        <v>100</v>
-      </c>
-      <c r="G33" s="14">
-        <v>100</v>
-      </c>
-      <c r="H33" s="14">
-        <v>100</v>
-      </c>
-      <c r="I33" s="14">
-        <v>100</v>
-      </c>
-      <c r="J33" s="14">
-        <v>100</v>
-      </c>
-      <c r="K33" s="14">
-        <v>100</v>
-      </c>
-      <c r="L33" s="14">
-        <v>100</v>
-      </c>
-      <c r="M33" s="15">
-        <v>100</v>
+      <c r="C33" s="12">
+        <v>4</v>
+      </c>
+      <c r="D33" s="12">
+        <v>4</v>
+      </c>
+      <c r="E33" s="12">
+        <v>4</v>
+      </c>
+      <c r="F33" s="12">
+        <v>4</v>
+      </c>
+      <c r="G33" s="12">
+        <v>4</v>
+      </c>
+      <c r="H33" s="12">
+        <v>4</v>
+      </c>
+      <c r="I33" s="12">
+        <v>4</v>
+      </c>
+      <c r="J33" s="12">
+        <v>4</v>
+      </c>
+      <c r="K33" s="12">
+        <v>4</v>
+      </c>
+      <c r="L33" s="12">
+        <v>4</v>
+      </c>
+      <c r="M33" s="12">
+        <v>4</v>
       </c>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.25">
@@ -1926,38 +1926,38 @@
       <c r="B34" s="16">
         <v>1000</v>
       </c>
-      <c r="C34" s="17">
-        <v>100</v>
-      </c>
-      <c r="D34" s="17">
-        <v>100</v>
-      </c>
-      <c r="E34" s="17">
-        <v>100</v>
-      </c>
-      <c r="F34" s="17">
-        <v>100</v>
-      </c>
-      <c r="G34" s="17">
-        <v>100</v>
-      </c>
-      <c r="H34" s="17">
-        <v>100</v>
-      </c>
-      <c r="I34" s="17">
-        <v>100</v>
-      </c>
-      <c r="J34" s="17">
-        <v>100</v>
-      </c>
-      <c r="K34" s="17">
-        <v>100</v>
-      </c>
-      <c r="L34" s="17">
-        <v>100</v>
-      </c>
-      <c r="M34" s="18">
-        <v>100</v>
+      <c r="C34" s="12">
+        <v>4</v>
+      </c>
+      <c r="D34" s="12">
+        <v>4</v>
+      </c>
+      <c r="E34" s="12">
+        <v>4</v>
+      </c>
+      <c r="F34" s="12">
+        <v>4</v>
+      </c>
+      <c r="G34" s="12">
+        <v>4</v>
+      </c>
+      <c r="H34" s="12">
+        <v>4</v>
+      </c>
+      <c r="I34" s="12">
+        <v>4</v>
+      </c>
+      <c r="J34" s="12">
+        <v>4</v>
+      </c>
+      <c r="K34" s="12">
+        <v>4</v>
+      </c>
+      <c r="L34" s="12">
+        <v>4</v>
+      </c>
+      <c r="M34" s="12">
+        <v>4</v>
       </c>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.25">

</xml_diff>